<commit_message>
update contractExport & contractImport, add field(ForeignTradeNum,InvoiceNum)
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/asset/contract/contractExport/APM_Contract_Export_Template.xlsx
+++ b/src/src/main/webapp/portal/asset/contract/contractExport/APM_Contract_Export_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{962663FF-4515-4E29-9A22-BC5D976AB590}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{102E080C-5613-48DE-91C1-A96184AB93A4}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>合同编号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -80,6 +80,14 @@
   </si>
   <si>
     <t>合同名称</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>外贸合同号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>发票号</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,21 +413,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.375" customWidth="1"/>
-    <col min="2" max="2" width="14.625" customWidth="1"/>
-    <col min="3" max="4" width="15.5" customWidth="1"/>
-    <col min="5" max="5" width="15.875" customWidth="1"/>
-    <col min="6" max="6" width="16.75" customWidth="1"/>
-    <col min="7" max="7" width="16.625" customWidth="1"/>
-    <col min="8" max="8" width="16.375" customWidth="1"/>
-    <col min="9" max="9" width="17.25" customWidth="1"/>
-    <col min="10" max="10" width="28.375" customWidth="1"/>
+    <col min="2" max="4" width="14.625" customWidth="1"/>
+    <col min="5" max="6" width="15.5" customWidth="1"/>
+    <col min="7" max="7" width="15.875" customWidth="1"/>
+    <col min="8" max="8" width="16.75" customWidth="1"/>
+    <col min="9" max="9" width="16.625" customWidth="1"/>
+    <col min="10" max="10" width="16.375" customWidth="1"/>
+    <col min="11" max="11" width="17.25" customWidth="1"/>
+    <col min="12" max="12" width="28.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -427,27 +435,33 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>